<commit_message>
publish: push certificate-demo (e9c2d50)
</commit_message>
<xml_diff>
--- a/preview/certificate-demo/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/preview/certificate-demo/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch certificate-demo · commit 34ac789 (built 2026-10-16 09:35 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch certificate-demo · commit e9c2d50 (built 2026-10-16 09:44 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit 34ac789 · built 2026-10-16 09:35 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7369,7 +7369,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit 34ac789 · built 2026-10-16 09:35 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12350,7 +12350,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit 34ac789 · built 2026-10-16 09:35 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14483,7 +14483,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit 34ac789 · built 2026-10-16 09:35 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27252,7 +27252,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit 34ac789 · built 2026-10-16 09:35 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28562,7 +28562,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit 34ac789 · built 2026-10-16 09:35 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29154,7 +29154,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit 34ac789 · built 2026-10-16 09:35 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32465,7 +32465,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit 34ac789 · built 2026-10-16 09:35 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33647,7 +33647,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit 34ac789 · built 2026-10-16 09:35 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35142,7 +35142,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit 34ac789 · built 2026-10-16 09:35 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37310,7 +37310,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit 34ac789 · built 2026-10-16 09:35 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42583,7 +42583,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit 34ac789 · built 2026-10-16 09:35 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46793,7 +46793,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit 34ac789 · built 2026-10-16 09:35 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>

<commit_message>
publish: push certificate-demo (e880b61)
</commit_message>
<xml_diff>
--- a/preview/certificate-demo/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/preview/certificate-demo/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch certificate-demo · commit e9c2d50 (built 2026-10-16 09:44 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch certificate-demo · commit e880b61 (built 2026-10-16 11:54 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7369,7 +7369,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12350,7 +12350,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14483,7 +14483,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27252,7 +27252,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28562,7 +28562,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29154,7 +29154,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32465,7 +32465,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33647,7 +33647,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35142,7 +35142,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37310,7 +37310,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42583,7 +42583,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46793,7 +46793,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e9c2d50 · built 2026-10-16 09:44 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>

<commit_message>
publish: push certificate-demo (f7bb10a)
</commit_message>
<xml_diff>
--- a/preview/certificate-demo/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/preview/certificate-demo/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch certificate-demo · commit e880b61 (built 2026-10-16 11:54 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch certificate-demo · commit f7bb10a (built 2026-10-16 12:59 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit f7bb10a · built 2026-10-16 12:59 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7369,7 +7369,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit f7bb10a · built 2026-10-16 12:59 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12350,7 +12350,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit f7bb10a · built 2026-10-16 12:59 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14483,7 +14483,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit f7bb10a · built 2026-10-16 12:59 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27252,7 +27252,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit f7bb10a · built 2026-10-16 12:59 PHT</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28562,7 +28562,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit f7bb10a · built 2026-10-16 12:59 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29154,7 +29154,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit f7bb10a · built 2026-10-16 12:59 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32465,7 +32465,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit f7bb10a · built 2026-10-16 12:59 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33647,7 +33647,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit f7bb10a · built 2026-10-16 12:59 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35142,7 +35142,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit f7bb10a · built 2026-10-16 12:59 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37310,7 +37310,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit f7bb10a · built 2026-10-16 12:59 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42583,7 +42583,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit f7bb10a · built 2026-10-16 12:59 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46793,7 +46793,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit e880b61 · built 2026-10-16 11:54 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch certificate-demo · commit f7bb10a · built 2026-10-16 12:59 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>